<commit_message>
updated with su rrogate model testing and evaluation (Gaussian Process)
</commit_message>
<xml_diff>
--- a/ImageJ gel analysis results_YI.xlsx
+++ b/ImageJ gel analysis results_YI.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jahanvisingh/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5439192F-5945-7647-BDD1-9AC369E83340}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{03C592E3-4253-AD4D-AD44-86F3B17BDBBF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="17160" yWindow="940" windowWidth="16880" windowHeight="19340" xr2:uid="{894A101D-5A18-4339-9A8B-9BDEF358C34E}"/>
+    <workbookView xWindow="17160" yWindow="940" windowWidth="16880" windowHeight="19360" xr2:uid="{894A101D-5A18-4339-9A8B-9BDEF358C34E}"/>
   </bookViews>
   <sheets>
-    <sheet name="6 × 10⁶ " sheetId="1" r:id="rId1"/>
+    <sheet name="sheet 1" sheetId="1" r:id="rId1"/>
     <sheet name="6 × 10⁴ " sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
@@ -940,43 +940,43 @@
     <xf numFmtId="0" fontId="26" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="22" fillId="34" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="23" fillId="34" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="34" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="23" fillId="34" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="34" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="23" fillId="34" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="34" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="23" fillId="34" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="23" fillId="34" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="34" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="23" fillId="34" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="23" fillId="34" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="34" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="34" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="34" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="34" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="34" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="34" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="34" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2335,13 +2335,13 @@
       <c r="J2" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="K2" s="33" t="s">
+      <c r="K2" s="23" t="s">
         <v>2</v>
       </c>
-      <c r="L2" s="33"/>
-      <c r="M2" s="33"/>
-      <c r="N2" s="33"/>
-      <c r="O2" s="33"/>
+      <c r="L2" s="23"/>
+      <c r="M2" s="23"/>
+      <c r="N2" s="23"/>
+      <c r="O2" s="23"/>
     </row>
     <row r="3" spans="1:15" ht="30.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="4">
@@ -2374,11 +2374,11 @@
       <c r="J3" s="16">
         <v>100</v>
       </c>
-      <c r="K3" s="23"/>
-      <c r="L3" s="23"/>
-      <c r="M3" s="23"/>
-      <c r="N3" s="23"/>
-      <c r="O3" s="23"/>
+      <c r="K3" s="24"/>
+      <c r="L3" s="24"/>
+      <c r="M3" s="24"/>
+      <c r="N3" s="24"/>
+      <c r="O3" s="24"/>
     </row>
     <row r="4" spans="1:15" ht="30.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="4">
@@ -2412,96 +2412,96 @@
         <f>(C4/C3)*100</f>
         <v>36.366141271189953</v>
       </c>
-      <c r="K4" s="23"/>
-      <c r="L4" s="23"/>
-      <c r="M4" s="23"/>
-      <c r="N4" s="23"/>
-      <c r="O4" s="23"/>
+      <c r="K4" s="24"/>
+      <c r="L4" s="24"/>
+      <c r="M4" s="24"/>
+      <c r="N4" s="24"/>
+      <c r="O4" s="24"/>
     </row>
     <row r="5" spans="1:15" ht="15.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="25"/>
-      <c r="B5" s="26"/>
-      <c r="C5" s="26"/>
-      <c r="D5" s="26"/>
-      <c r="E5" s="26"/>
-      <c r="F5" s="26"/>
-      <c r="G5" s="26"/>
-      <c r="H5" s="26"/>
-      <c r="I5" s="26"/>
-      <c r="J5" s="34"/>
-      <c r="K5" s="23"/>
-      <c r="L5" s="23"/>
-      <c r="M5" s="23"/>
-      <c r="N5" s="23"/>
-      <c r="O5" s="23"/>
+      <c r="A5" s="28"/>
+      <c r="B5" s="29"/>
+      <c r="C5" s="29"/>
+      <c r="D5" s="29"/>
+      <c r="E5" s="29"/>
+      <c r="F5" s="29"/>
+      <c r="G5" s="29"/>
+      <c r="H5" s="29"/>
+      <c r="I5" s="29"/>
+      <c r="J5" s="30"/>
+      <c r="K5" s="24"/>
+      <c r="L5" s="24"/>
+      <c r="M5" s="24"/>
+      <c r="N5" s="24"/>
+      <c r="O5" s="24"/>
     </row>
     <row r="6" spans="1:15" ht="15.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="27"/>
-      <c r="B6" s="28"/>
-      <c r="C6" s="28"/>
-      <c r="D6" s="28"/>
-      <c r="E6" s="28"/>
-      <c r="F6" s="28"/>
-      <c r="G6" s="28"/>
-      <c r="H6" s="28"/>
-      <c r="I6" s="28"/>
-      <c r="J6" s="35"/>
-      <c r="K6" s="23"/>
-      <c r="L6" s="23"/>
-      <c r="M6" s="23"/>
-      <c r="N6" s="23"/>
-      <c r="O6" s="23"/>
+      <c r="A6" s="31"/>
+      <c r="B6" s="32"/>
+      <c r="C6" s="32"/>
+      <c r="D6" s="32"/>
+      <c r="E6" s="32"/>
+      <c r="F6" s="32"/>
+      <c r="G6" s="32"/>
+      <c r="H6" s="32"/>
+      <c r="I6" s="32"/>
+      <c r="J6" s="33"/>
+      <c r="K6" s="24"/>
+      <c r="L6" s="24"/>
+      <c r="M6" s="24"/>
+      <c r="N6" s="24"/>
+      <c r="O6" s="24"/>
     </row>
     <row r="7" spans="1:15" ht="19.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="27"/>
-      <c r="B7" s="28"/>
-      <c r="C7" s="28"/>
-      <c r="D7" s="28"/>
-      <c r="E7" s="28"/>
-      <c r="F7" s="28"/>
-      <c r="G7" s="28"/>
-      <c r="H7" s="28"/>
-      <c r="I7" s="28"/>
-      <c r="J7" s="35"/>
-      <c r="K7" s="23"/>
-      <c r="L7" s="23"/>
-      <c r="M7" s="23"/>
-      <c r="N7" s="23"/>
-      <c r="O7" s="23"/>
+      <c r="A7" s="31"/>
+      <c r="B7" s="32"/>
+      <c r="C7" s="32"/>
+      <c r="D7" s="32"/>
+      <c r="E7" s="32"/>
+      <c r="F7" s="32"/>
+      <c r="G7" s="32"/>
+      <c r="H7" s="32"/>
+      <c r="I7" s="32"/>
+      <c r="J7" s="33"/>
+      <c r="K7" s="24"/>
+      <c r="L7" s="24"/>
+      <c r="M7" s="24"/>
+      <c r="N7" s="24"/>
+      <c r="O7" s="24"/>
     </row>
     <row r="8" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="29"/>
-      <c r="B8" s="30"/>
-      <c r="C8" s="30"/>
-      <c r="D8" s="30"/>
-      <c r="E8" s="30"/>
-      <c r="F8" s="30"/>
-      <c r="G8" s="30"/>
-      <c r="H8" s="30"/>
-      <c r="I8" s="30"/>
+      <c r="A8" s="34"/>
+      <c r="B8" s="35"/>
+      <c r="C8" s="35"/>
+      <c r="D8" s="35"/>
+      <c r="E8" s="35"/>
+      <c r="F8" s="35"/>
+      <c r="G8" s="35"/>
+      <c r="H8" s="35"/>
+      <c r="I8" s="35"/>
       <c r="J8" s="36"/>
-      <c r="K8" s="23"/>
-      <c r="L8" s="23"/>
-      <c r="M8" s="23"/>
-      <c r="N8" s="23"/>
-      <c r="O8" s="23"/>
+      <c r="K8" s="24"/>
+      <c r="L8" s="24"/>
+      <c r="M8" s="24"/>
+      <c r="N8" s="24"/>
+      <c r="O8" s="24"/>
     </row>
     <row r="9" spans="1:15" ht="16" x14ac:dyDescent="0.2">
-      <c r="A9" s="24"/>
-      <c r="B9" s="31"/>
-      <c r="C9" s="31"/>
-      <c r="D9" s="31"/>
-      <c r="E9" s="31"/>
-      <c r="F9" s="31"/>
-      <c r="G9" s="31"/>
-      <c r="H9" s="31"/>
-      <c r="I9" s="31"/>
-      <c r="J9" s="31"/>
-      <c r="K9" s="31"/>
-      <c r="L9" s="31"/>
-      <c r="M9" s="31"/>
-      <c r="N9" s="31"/>
-      <c r="O9" s="32"/>
+      <c r="A9" s="25"/>
+      <c r="B9" s="26"/>
+      <c r="C9" s="26"/>
+      <c r="D9" s="26"/>
+      <c r="E9" s="26"/>
+      <c r="F9" s="26"/>
+      <c r="G9" s="26"/>
+      <c r="H9" s="26"/>
+      <c r="I9" s="26"/>
+      <c r="J9" s="26"/>
+      <c r="K9" s="26"/>
+      <c r="L9" s="26"/>
+      <c r="M9" s="26"/>
+      <c r="N9" s="26"/>
+      <c r="O9" s="27"/>
     </row>
     <row r="10" spans="1:15" ht="39" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="4">
@@ -2723,11 +2723,11 @@
       <c r="J15" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="K15" s="23"/>
-      <c r="L15" s="23"/>
-      <c r="M15" s="23"/>
-      <c r="N15" s="23"/>
-      <c r="O15" s="23"/>
+      <c r="K15" s="24"/>
+      <c r="L15" s="24"/>
+      <c r="M15" s="24"/>
+      <c r="N15" s="24"/>
+      <c r="O15" s="24"/>
     </row>
     <row r="16" spans="1:15" ht="34" x14ac:dyDescent="0.2">
       <c r="A16" s="4">
@@ -2761,64 +2761,64 @@
         <f>(C16/C10)*100</f>
         <v>13.068928024029573</v>
       </c>
-      <c r="K16" s="23"/>
-      <c r="L16" s="23"/>
-      <c r="M16" s="23"/>
-      <c r="N16" s="23"/>
-      <c r="O16" s="23"/>
+      <c r="K16" s="24"/>
+      <c r="L16" s="24"/>
+      <c r="M16" s="24"/>
+      <c r="N16" s="24"/>
+      <c r="O16" s="24"/>
     </row>
     <row r="17" spans="1:15" ht="15.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="23" t="s">
+      <c r="A17" s="24" t="s">
         <v>28</v>
       </c>
-      <c r="B17" s="23"/>
-      <c r="C17" s="23"/>
-      <c r="D17" s="23"/>
-      <c r="E17" s="23"/>
-      <c r="F17" s="23"/>
-      <c r="G17" s="23"/>
-      <c r="H17" s="23"/>
-      <c r="I17" s="23"/>
-      <c r="J17" s="23"/>
-      <c r="K17" s="23"/>
-      <c r="L17" s="23"/>
-      <c r="M17" s="23"/>
-      <c r="N17" s="23"/>
-      <c r="O17" s="23"/>
+      <c r="B17" s="24"/>
+      <c r="C17" s="24"/>
+      <c r="D17" s="24"/>
+      <c r="E17" s="24"/>
+      <c r="F17" s="24"/>
+      <c r="G17" s="24"/>
+      <c r="H17" s="24"/>
+      <c r="I17" s="24"/>
+      <c r="J17" s="24"/>
+      <c r="K17" s="24"/>
+      <c r="L17" s="24"/>
+      <c r="M17" s="24"/>
+      <c r="N17" s="24"/>
+      <c r="O17" s="24"/>
     </row>
     <row r="18" spans="1:15" ht="15.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="23"/>
-      <c r="B18" s="23"/>
-      <c r="C18" s="23"/>
-      <c r="D18" s="23"/>
-      <c r="E18" s="23"/>
-      <c r="F18" s="23"/>
-      <c r="G18" s="23"/>
-      <c r="H18" s="23"/>
-      <c r="I18" s="23"/>
-      <c r="J18" s="23"/>
-      <c r="K18" s="23"/>
-      <c r="L18" s="23"/>
-      <c r="M18" s="23"/>
-      <c r="N18" s="23"/>
-      <c r="O18" s="23"/>
+      <c r="A18" s="24"/>
+      <c r="B18" s="24"/>
+      <c r="C18" s="24"/>
+      <c r="D18" s="24"/>
+      <c r="E18" s="24"/>
+      <c r="F18" s="24"/>
+      <c r="G18" s="24"/>
+      <c r="H18" s="24"/>
+      <c r="I18" s="24"/>
+      <c r="J18" s="24"/>
+      <c r="K18" s="24"/>
+      <c r="L18" s="24"/>
+      <c r="M18" s="24"/>
+      <c r="N18" s="24"/>
+      <c r="O18" s="24"/>
     </row>
     <row r="19" spans="1:15" ht="15.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="23"/>
-      <c r="B19" s="23"/>
-      <c r="C19" s="23"/>
-      <c r="D19" s="23"/>
-      <c r="E19" s="23"/>
-      <c r="F19" s="23"/>
-      <c r="G19" s="23"/>
-      <c r="H19" s="23"/>
-      <c r="I19" s="23"/>
-      <c r="J19" s="23"/>
-      <c r="K19" s="23"/>
-      <c r="L19" s="23"/>
-      <c r="M19" s="23"/>
-      <c r="N19" s="23"/>
-      <c r="O19" s="23"/>
+      <c r="A19" s="24"/>
+      <c r="B19" s="24"/>
+      <c r="C19" s="24"/>
+      <c r="D19" s="24"/>
+      <c r="E19" s="24"/>
+      <c r="F19" s="24"/>
+      <c r="G19" s="24"/>
+      <c r="H19" s="24"/>
+      <c r="I19" s="24"/>
+      <c r="J19" s="24"/>
+      <c r="K19" s="24"/>
+      <c r="L19" s="24"/>
+      <c r="M19" s="24"/>
+      <c r="N19" s="24"/>
+      <c r="O19" s="24"/>
     </row>
   </sheetData>
   <mergeCells count="6">

</xml_diff>